<commit_message>
feat: update OFI dashboards and operational visualizations
</commit_message>
<xml_diff>
--- a/dados/SURVEY_CBO.xlsx
+++ b/dados/SURVEY_CBO.xlsx
@@ -1,33 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="988" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO ALESSANDRA" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO ALIANCA" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO ANITA" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO ARPOADOR" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO CAMPOS" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO CAROLINA" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO COPACABANA" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO ENERGY" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO FLAMENGO" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO IPANEMA" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO ISABELLA" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO ITAJAI" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO MANOELLA" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO OCEANA" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO RENATA" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO RIO" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO SUPPORTER" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO VITORIA" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO WAVE" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBO WISER" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DELTA CARDINAL" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DELTA COMMANDER" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="CBO ALESSANDRA" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CBO ALIANCA" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="CBO ANITA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CBO ARPOADOR" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CBO CAMPOS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="CBO CAROLINA" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CBO COPACABANA" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="CBO ENERGY" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="CBO FLAMENGO" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="CBO IPANEMA" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="CBO ISABELLA" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="CBO ITAJAI" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="CBO MANOELLA" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="CBO OCEANA" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="CBO RENATA" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="CBO RIO" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="CBO SUPPORTER" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="CBO VITORIA" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="CBO WAVE" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="CBO WISER" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="DELTA CARDINAL" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="DELTA COMMANDER" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'CBO ALESSANDRA'!$A$1:$S$1</definedName>
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34.5703125" customWidth="1" min="1" max="1"/>
@@ -1137,9 +1137,6 @@
       <c r="A24" s="18" t="n">
         <v>46237.32916666667</v>
       </c>
-      <c r="B24" t="n">
-        <v/>
-      </c>
       <c r="M24" t="n">
         <v>-22.841309</v>
       </c>
@@ -1149,12 +1146,28 @@
       <c r="Q24" s="18" t="n">
         <v>46237.32777777778</v>
       </c>
-      <c r="R24" t="n">
-        <v/>
-      </c>
       <c r="S24" t="inlineStr">
         <is>
           <t>At Anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>46278.86458333334</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-24.640833</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-42.195835</v>
+      </c>
+      <c r="Q25" s="18" t="n">
+        <v>46277.17361111111</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Underway using Engine</t>
         </is>
       </c>
     </row>
@@ -1170,7 +1183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="13.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="20.5703125" customWidth="1" min="1" max="1"/>
@@ -1791,9 +1804,6 @@
       <c r="A24" s="18" t="n">
         <v>46237.32916666667</v>
       </c>
-      <c r="B24" t="n">
-        <v/>
-      </c>
       <c r="M24" t="n">
         <v>-23.524544</v>
       </c>
@@ -1803,12 +1813,28 @@
       <c r="Q24" s="18" t="n">
         <v>46237.15555555555</v>
       </c>
-      <c r="R24" t="n">
-        <v/>
-      </c>
       <c r="S24" t="inlineStr">
         <is>
           <t>Stopped</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>46278.86458333334</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-23.549366</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-41.096352</v>
+      </c>
+      <c r="Q25" s="18" t="n">
+        <v>46277.02430555555</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Underway using Engine</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29.140625" customWidth="1" min="1" max="1"/>
@@ -2438,9 +2464,6 @@
       <c r="A24" s="18" t="n">
         <v>46237.33055555556</v>
       </c>
-      <c r="B24" t="n">
-        <v/>
-      </c>
       <c r="M24" t="n">
         <v>-22.894377</v>
       </c>
@@ -2450,12 +2473,28 @@
       <c r="Q24" s="18" t="n">
         <v>46237.32083333333</v>
       </c>
-      <c r="R24" t="n">
-        <v/>
-      </c>
       <c r="S24" t="inlineStr">
         <is>
           <t>Moored</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>46278.85138888889</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-22.222944</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-40.309349</v>
+      </c>
+      <c r="Q25" s="18" t="n">
+        <v>46278.43819444445</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Underway using Engine</t>
         </is>
       </c>
     </row>
@@ -2470,7 +2509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23.42578125" customWidth="1" min="1" max="1"/>
@@ -3079,9 +3118,6 @@
       <c r="A24" s="18" t="n">
         <v>46237.33055555556</v>
       </c>
-      <c r="B24" t="n">
-        <v/>
-      </c>
       <c r="M24" t="n">
         <v>-22.825138</v>
       </c>
@@ -3091,12 +3127,28 @@
       <c r="Q24" s="18" t="n">
         <v>46237.32083333333</v>
       </c>
-      <c r="R24" t="n">
-        <v/>
-      </c>
       <c r="S24" t="inlineStr">
         <is>
           <t>At Anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>46278.85138888889</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-21.241184</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-40.035839</v>
+      </c>
+      <c r="Q25" s="18" t="n">
+        <v>46278.33055555556</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Restricted Manoeuvrability</t>
         </is>
       </c>
     </row>
@@ -3111,7 +3163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3727,9 +3779,6 @@
       <c r="A24" s="18" t="n">
         <v>46237.33055555556</v>
       </c>
-      <c r="B24" t="n">
-        <v/>
-      </c>
       <c r="M24" t="n">
         <v>-22.881086</v>
       </c>
@@ -3739,10 +3788,26 @@
       <c r="Q24" s="18" t="n">
         <v>46237.32708333333</v>
       </c>
-      <c r="R24" t="n">
-        <v/>
-      </c>
       <c r="S24" t="inlineStr">
+        <is>
+          <t>Moored</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>46278.85138888889</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-21.864485</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-41.016666</v>
+      </c>
+      <c r="Q25" s="18" t="n">
+        <v>46278.84722222222</v>
+      </c>
+      <c r="S25" t="inlineStr">
         <is>
           <t>Moored</t>
         </is>
@@ -3759,7 +3824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24.7109375" customWidth="1" min="1" max="1"/>
@@ -4371,9 +4436,6 @@
       <c r="A24" s="18" t="n">
         <v>46237.33055555556</v>
       </c>
-      <c r="B24" t="n">
-        <v/>
-      </c>
       <c r="M24" t="n">
         <v>-22.841206</v>
       </c>
@@ -4383,12 +4445,28 @@
       <c r="Q24" s="18" t="n">
         <v>46237.32430555556</v>
       </c>
-      <c r="R24" t="n">
-        <v/>
-      </c>
       <c r="S24" t="inlineStr">
         <is>
           <t>At Anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>46278.85138888889</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-25.021685</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-42.66824</v>
+      </c>
+      <c r="Q25" s="18" t="n">
+        <v>46277.43125</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Stopped</t>
         </is>
       </c>
     </row>
@@ -4403,7 +4481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29.5703125" customWidth="1" min="1" max="1"/>
@@ -5028,9 +5106,6 @@
       <c r="A24" s="18" t="n">
         <v>46237.33055555556</v>
       </c>
-      <c r="B24" t="n">
-        <v/>
-      </c>
       <c r="M24" t="n">
         <v>-21.205</v>
       </c>
@@ -5040,10 +5115,26 @@
       <c r="Q24" s="18" t="n">
         <v>46234.74513888889</v>
       </c>
-      <c r="R24" t="n">
-        <v/>
-      </c>
       <c r="S24" t="inlineStr">
+        <is>
+          <t>Stopped</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>46278.85138888889</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-21.214226</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-39.997829</v>
+      </c>
+      <c r="Q25" s="18" t="n">
+        <v>46278.33333333334</v>
+      </c>
+      <c r="S25" t="inlineStr">
         <is>
           <t>Stopped</t>
         </is>
@@ -5060,7 +5151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24.140625" customWidth="1" min="1" max="1"/>
@@ -5669,9 +5760,6 @@
       <c r="A24" s="18" t="n">
         <v>46237.33055555556</v>
       </c>
-      <c r="B24" t="n">
-        <v/>
-      </c>
       <c r="M24" t="n">
         <v>-30.372272</v>
       </c>
@@ -5681,10 +5769,26 @@
       <c r="Q24" s="18" t="n">
         <v>44677.81111111111</v>
       </c>
-      <c r="R24" t="n">
-        <v/>
-      </c>
       <c r="S24" t="inlineStr">
+        <is>
+          <t>Class B</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>46278.85138888889</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-30.372272</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-47.695133</v>
+      </c>
+      <c r="Q25" s="18" t="n">
+        <v>44677.81111111111</v>
+      </c>
+      <c r="S25" t="inlineStr">
         <is>
           <t>Class B</t>
         </is>
@@ -5701,7 +5805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -6314,9 +6418,6 @@
       <c r="A24" s="18" t="n">
         <v>46237.33055555556</v>
       </c>
-      <c r="B24" t="n">
-        <v/>
-      </c>
       <c r="M24" t="n">
         <v>-22.479593</v>
       </c>
@@ -6326,10 +6427,26 @@
       <c r="Q24" s="18" t="n">
         <v>46237.32777777778</v>
       </c>
-      <c r="R24" t="n">
-        <v/>
-      </c>
       <c r="S24" t="inlineStr">
+        <is>
+          <t>Underway using Engine</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>46278.85138888889</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-22.413794</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-40.920341</v>
+      </c>
+      <c r="Q25" s="18" t="n">
+        <v>46278.65694444445</v>
+      </c>
+      <c r="S25" t="inlineStr">
         <is>
           <t>Underway using Engine</t>
         </is>
@@ -6346,7 +6463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30.28515625" customWidth="1" min="1" max="1"/>
@@ -6955,9 +7072,6 @@
       <c r="A24" s="18" t="n">
         <v>46237.33055555556</v>
       </c>
-      <c r="B24" t="n">
-        <v/>
-      </c>
       <c r="M24" t="n">
         <v>-22.864527</v>
       </c>
@@ -6967,10 +7081,26 @@
       <c r="Q24" s="18" t="n">
         <v>45839.57638888889</v>
       </c>
-      <c r="R24" t="n">
-        <v/>
-      </c>
       <c r="S24" t="inlineStr">
+        <is>
+          <t>Moored</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>46278.85138888889</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-22.864527</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-43.111076</v>
+      </c>
+      <c r="Q25" s="18" t="n">
+        <v>45839.57638888889</v>
+      </c>
+      <c r="S25" t="inlineStr">
         <is>
           <t>Moored</t>
         </is>
@@ -6987,7 +7117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24.85546875" customWidth="1" min="1" max="1"/>
@@ -7596,9 +7726,6 @@
       <c r="A24" s="18" t="n">
         <v>46237.33055555556</v>
       </c>
-      <c r="B24" t="n">
-        <v/>
-      </c>
       <c r="M24" t="n">
         <v>-24.652611</v>
       </c>
@@ -7608,10 +7735,26 @@
       <c r="Q24" s="18" t="n">
         <v>46237.03888888889</v>
       </c>
-      <c r="R24" t="n">
-        <v/>
-      </c>
       <c r="S24" t="inlineStr">
+        <is>
+          <t>Restricted Manoeuvrability</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>46278.85138888889</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-24.653959</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-42.235405</v>
+      </c>
+      <c r="Q25" s="18" t="n">
+        <v>46277.15972222222</v>
+      </c>
+      <c r="S25" t="inlineStr">
         <is>
           <t>Restricted Manoeuvrability</t>
         </is>
@@ -7628,7 +7771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29.28515625" customWidth="1" min="1" max="1"/>
@@ -8242,9 +8385,6 @@
       <c r="A24" s="18" t="n">
         <v>46237.32916666667</v>
       </c>
-      <c r="B24" t="n">
-        <v/>
-      </c>
       <c r="M24" t="n">
         <v>-22.384466</v>
       </c>
@@ -8254,12 +8394,28 @@
       <c r="Q24" s="18" t="n">
         <v>46237.32777777778</v>
       </c>
-      <c r="R24" t="n">
-        <v/>
-      </c>
       <c r="S24" t="inlineStr">
         <is>
           <t>Moored</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>46278.86458333334</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-25.570738</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-42.842857</v>
+      </c>
+      <c r="Q25" s="18" t="n">
+        <v>46277.42777777778</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Underway using Engine</t>
         </is>
       </c>
     </row>
@@ -8275,7 +8431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20.28515625" customWidth="1" min="1" max="1"/>
@@ -8890,9 +9046,6 @@
       <c r="A24" s="18" t="n">
         <v>46237.33055555556</v>
       </c>
-      <c r="B24" t="n">
-        <v/>
-      </c>
       <c r="M24" t="n">
         <v>-21.854759</v>
       </c>
@@ -8902,12 +9055,28 @@
       <c r="Q24" s="18" t="n">
         <v>46237.32708333333</v>
       </c>
-      <c r="R24" t="n">
-        <v/>
-      </c>
       <c r="S24" t="inlineStr">
         <is>
           <t>Moored</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>46278.85138888889</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-23.597019</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-42.626418</v>
+      </c>
+      <c r="Q25" s="18" t="n">
+        <v>46278.84513888889</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Underway using Engine</t>
         </is>
       </c>
     </row>
@@ -8922,7 +9091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28.140625" customWidth="1" min="1" max="1"/>
@@ -9534,9 +9703,6 @@
       <c r="A24" s="18" t="n">
         <v>46237.33055555556</v>
       </c>
-      <c r="B24" t="n">
-        <v/>
-      </c>
       <c r="M24" t="n">
         <v>-22.854086</v>
       </c>
@@ -9546,12 +9712,28 @@
       <c r="Q24" s="18" t="n">
         <v>46237.32152777778</v>
       </c>
-      <c r="R24" t="n">
-        <v/>
-      </c>
       <c r="S24" t="inlineStr">
         <is>
           <t>At Anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>46278.85138888889</v>
+      </c>
+      <c r="M25" t="n">
+        <v>7.216545</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-55.740231</v>
+      </c>
+      <c r="Q25" s="18" t="n">
+        <v>46278.84583333333</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Underway using Engine</t>
         </is>
       </c>
     </row>
@@ -9566,7 +9748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24.42578125" customWidth="1" min="1" max="1"/>
@@ -10183,9 +10365,6 @@
       <c r="A24" s="18" t="n">
         <v>46237.33055555556</v>
       </c>
-      <c r="B24" t="n">
-        <v/>
-      </c>
       <c r="M24" t="n">
         <v>-22.846739</v>
       </c>
@@ -10195,12 +10374,28 @@
       <c r="Q24" s="18" t="n">
         <v>46237.32152777778</v>
       </c>
-      <c r="R24" t="n">
-        <v/>
-      </c>
       <c r="S24" t="inlineStr">
         <is>
           <t>At Anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>46278.85138888889</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-22.027397</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-40.713665</v>
+      </c>
+      <c r="Q25" s="18" t="n">
+        <v>46278.05902777778</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Underway using Engine</t>
         </is>
       </c>
     </row>
@@ -10215,7 +10410,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI36"/>
+  <dimension ref="A1:AI37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23.5703125" customWidth="1" min="1" max="1"/>
@@ -11716,9 +11911,6 @@
       <c r="A36" s="18" t="n">
         <v>46237.32916666667</v>
       </c>
-      <c r="B36" t="n">
-        <v/>
-      </c>
       <c r="M36" t="n">
         <v>-23.561159</v>
       </c>
@@ -11728,12 +11920,28 @@
       <c r="Q36" s="18" t="n">
         <v>46237.06319444445</v>
       </c>
-      <c r="R36" t="n">
-        <v/>
-      </c>
       <c r="S36" t="inlineStr">
         <is>
           <t>Stopped</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="18" t="n">
+        <v>46278.86458333334</v>
+      </c>
+      <c r="M37" t="n">
+        <v>-23.098541</v>
+      </c>
+      <c r="N37" t="n">
+        <v>-42.777458</v>
+      </c>
+      <c r="Q37" s="18" t="n">
+        <v>46277.86597222222</v>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>Underway using Engine</t>
         </is>
       </c>
     </row>
@@ -11749,7 +11957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S48"/>
+  <dimension ref="A1:S49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28.5703125" customWidth="1" min="1" max="1"/>
@@ -13984,9 +14192,6 @@
       <c r="A48" s="18" t="n">
         <v>46237.32916666667</v>
       </c>
-      <c r="B48" t="n">
-        <v/>
-      </c>
       <c r="M48" t="n">
         <v>-24.637222</v>
       </c>
@@ -13996,12 +14201,28 @@
       <c r="Q48" s="18" t="n">
         <v>46236.76388888889</v>
       </c>
-      <c r="R48" t="n">
-        <v/>
-      </c>
       <c r="S48" t="inlineStr">
         <is>
           <t>Stopped</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="18" t="n">
+        <v>46278.86458333334</v>
+      </c>
+      <c r="M49" t="n">
+        <v>-24.659252</v>
+      </c>
+      <c r="N49" t="n">
+        <v>-42.457294</v>
+      </c>
+      <c r="Q49" s="18" t="n">
+        <v>46275.42083333333</v>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>Underway using Engine</t>
         </is>
       </c>
     </row>
@@ -14016,7 +14237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33.42578125" customWidth="1" min="1" max="1"/>
@@ -14629,9 +14850,6 @@
       <c r="A24" s="18" t="n">
         <v>46237.32916666667</v>
       </c>
-      <c r="B24" t="n">
-        <v/>
-      </c>
       <c r="M24" t="n">
         <v>-22.864473</v>
       </c>
@@ -14641,10 +14859,26 @@
       <c r="Q24" s="18" t="n">
         <v>44390.56527777778</v>
       </c>
-      <c r="R24" t="n">
-        <v/>
-      </c>
       <c r="S24" t="inlineStr">
+        <is>
+          <t>Moored</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>46278.86458333334</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-22.864473</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-43.109585</v>
+      </c>
+      <c r="Q25" s="18" t="n">
+        <v>44390.56527777778</v>
+      </c>
+      <c r="S25" t="inlineStr">
         <is>
           <t>Moored</t>
         </is>
@@ -14661,7 +14895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38.7109375" customWidth="1" min="1" max="1"/>
@@ -15276,9 +15510,6 @@
       <c r="A24" s="18" t="n">
         <v>46237.32916666667</v>
       </c>
-      <c r="B24" t="n">
-        <v/>
-      </c>
       <c r="M24" t="n">
         <v>-24.041594</v>
       </c>
@@ -15288,12 +15519,28 @@
       <c r="Q24" s="18" t="n">
         <v>46237.07291666666</v>
       </c>
-      <c r="R24" t="n">
-        <v/>
-      </c>
       <c r="S24" t="inlineStr">
         <is>
           <t>Underway using Engine</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>46278.86458333334</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-22.881845</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-43.117619</v>
+      </c>
+      <c r="Q25" s="18" t="n">
+        <v>46278.84444444445</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Moored</t>
         </is>
       </c>
     </row>
@@ -15308,7 +15555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S26"/>
+  <dimension ref="A1:S27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.28515625" customWidth="1" min="1" max="1"/>
@@ -16130,9 +16377,6 @@
       <c r="A26" s="18" t="n">
         <v>46237.32916666667</v>
       </c>
-      <c r="B26" t="n">
-        <v/>
-      </c>
       <c r="M26" t="n">
         <v>-22.844997</v>
       </c>
@@ -16142,18 +16386,34 @@
       <c r="Q26" s="18" t="n">
         <v>46237.32222222222</v>
       </c>
-      <c r="R26" t="n">
-        <v/>
-      </c>
       <c r="S26" t="inlineStr">
         <is>
           <t>Stopped</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="18" t="n">
+        <v>46278.86458333334</v>
+      </c>
+      <c r="M27" t="n">
+        <v>-22.894632</v>
+      </c>
+      <c r="N27" t="n">
+        <v>-43.212166</v>
+      </c>
+      <c r="Q27" s="18" t="n">
+        <v>46278.84305555555</v>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Moored</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:S19">
-    <filterColumn colId="18">
+    <filterColumn colId="18" hiddenButton="0" showButton="1">
       <filters>
         <filter val="moored"/>
       </filters>
@@ -16169,7 +16429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S25"/>
+  <dimension ref="A1:S26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -16814,9 +17074,6 @@
       <c r="A25" s="18" t="n">
         <v>46237.32916666667</v>
       </c>
-      <c r="B25" t="n">
-        <v/>
-      </c>
       <c r="M25" t="n">
         <v>-25.536068</v>
       </c>
@@ -16826,12 +17083,28 @@
       <c r="Q25" s="18" t="n">
         <v>46237.06319444445</v>
       </c>
-      <c r="R25" t="n">
-        <v/>
-      </c>
       <c r="S25" t="inlineStr">
         <is>
           <t>Restricted Manoeuvrability</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="n">
+        <v>46278.86458333334</v>
+      </c>
+      <c r="M26" t="n">
+        <v>-22.848885</v>
+      </c>
+      <c r="N26" t="n">
+        <v>-43.143326</v>
+      </c>
+      <c r="Q26" s="18" t="n">
+        <v>46278.84513888889</v>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>At Anchor</t>
         </is>
       </c>
     </row>
@@ -16846,7 +17119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.5703125" customWidth="1" min="1" max="1"/>
@@ -17467,9 +17740,6 @@
       <c r="A24" s="18" t="n">
         <v>46237.32916666667</v>
       </c>
-      <c r="B24" t="n">
-        <v/>
-      </c>
       <c r="M24" t="n">
         <v>-21.866407</v>
       </c>
@@ -17479,12 +17749,28 @@
       <c r="Q24" s="18" t="n">
         <v>46237.32430555556</v>
       </c>
-      <c r="R24" t="n">
-        <v/>
-      </c>
       <c r="S24" t="inlineStr">
         <is>
           <t>Moored</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>46278.86458333334</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-21.924328</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-39.756535</v>
+      </c>
+      <c r="Q25" s="18" t="n">
+        <v>46277.69722222222</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Underway using Engine</t>
         </is>
       </c>
     </row>

</xml_diff>